<commit_message>
Simplify Companies directory and link search strategy targets
</commit_message>
<xml_diff>
--- a/public/templates/xqtiv-company-import.xlsx
+++ b/public/templates/xqtiv-company-import.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies" sheetId="1" r:id="Rf5d099312a294eca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R16eb7e7faf174215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies" sheetId="1" r:id="R9a0f7501f00d4662"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R693e28e0962745d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -39,7 +39,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -56,6 +56,11 @@
         <x:fgColor rgb="FFFFF9E8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF002050"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -63,7 +68,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="11">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -74,6 +79,11 @@
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -289,9 +299,13 @@
     <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="38" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="38" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="28" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="28" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
+    <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="4" t="str">
         <x:v>Company</x:v>
       </x:c>
@@ -330,6 +344,18 @@
       </x:c>
       <x:c r="M1" s="4" t="str">
         <x:v>Notes</x:v>
+      </x:c>
+      <x:c r="N1" s="9" t="str">
+        <x:v>Sector</x:v>
+      </x:c>
+      <x:c r="O1" s="9" t="str">
+        <x:v>Subsector</x:v>
+      </x:c>
+      <x:c r="P1" s="9" t="str">
+        <x:v>Company size</x:v>
+      </x:c>
+      <x:c r="Q1" s="9" t="str">
+        <x:v>Revenue Band (USD)</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
@@ -979,6 +1005,50 @@
       <x:c r="C33" s="1"/>
       <x:c r="D33" s="1"/>
     </x:row>
+    <x:row r="35" ht="30" customHeight="1">
+      <x:c r="A35" s="1" t="str">
+        <x:v>Sector</x:v>
+      </x:c>
+      <x:c r="B35" s="1" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="C35" s="10" t="str">
+        <x:v>Business sector</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="30" customHeight="1">
+      <x:c r="A36" s="1" t="str">
+        <x:v>Subsector</x:v>
+      </x:c>
+      <x:c r="B36" s="1" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="C36" s="10" t="str">
+        <x:v>Business subsector</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="30" customHeight="1">
+      <x:c r="A37" s="1" t="str">
+        <x:v>Company size</x:v>
+      </x:c>
+      <x:c r="B37" s="1" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="C37" s="10" t="str">
+        <x:v>Use the employee bands listed in Companies.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="A38" s="1" t="str">
+        <x:v>Revenue Band (USD)</x:v>
+      </x:c>
+      <x:c r="B38" s="1" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="C38" s="10" t="str">
+        <x:v>Use the revenue bands listed in Companies.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>